<commit_message>
excel import is Done
</commit_message>
<xml_diff>
--- a/xlsx/asset_import_template (1).xlsx
+++ b/xlsx/asset_import_template (1).xlsx
@@ -20,36 +20,36 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
-  <si>
-    <t xml:space="preserve">name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">inventory_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">serial_number</t>
-  </si>
-  <si>
-    <t xml:space="preserve">quantity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">comment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">date_issue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">date_purchasing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">next_service</t>
-  </si>
-  <si>
-    <t xml:space="preserve">service_period</t>
-  </si>
-  <si>
-    <t xml:space="preserve">check_period</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+  <si>
+    <t xml:space="preserve">Название</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Инвентарный номер</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Серийный номер</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Количество</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Комментарий</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дата выпуска</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дата покупки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дата обслуживания</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Период обслуживания</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Период проверки</t>
   </si>
   <si>
     <t xml:space="preserve">Ноутбук Dell Latitude 5520</t>
@@ -61,18 +61,6 @@
     <t xml:space="preserve">SN987654321</t>
   </si>
   <si>
-    <t xml:space="preserve">Выдан сотруднику отдела разработки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-10-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-09-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-10-01</t>
-  </si>
-  <si>
     <t xml:space="preserve">СМЕННАЯ ПРЕСС-ФОРМУ ПОДСТАВКА НА ТРЕВЕРСЕГЛАВНОГО КАТАЛИЗАТОРА </t>
   </si>
   <si>
@@ -82,15 +70,6 @@
     <t xml:space="preserve">проверка excel 1</t>
   </si>
   <si>
-    <t xml:space="preserve">2023-10-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-09-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-10-02</t>
-  </si>
-  <si>
     <t xml:space="preserve">Производственный общий </t>
   </si>
   <si>
@@ -100,37 +79,20 @@
     <t xml:space="preserve">проверка excel 2</t>
   </si>
   <si>
-    <t xml:space="preserve">2023-10-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-09-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-10-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сварочный цех</t>
-  </si>
-  <si>
-    <t xml:space="preserve">проверка excel 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-10-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-09-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-10-04</t>
+    <t xml:space="preserve">ПО \"Автовесовая\" Организация движения</t>
+  </si>
+  <si>
+    <t xml:space="preserve">проверка excel 44444</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="@"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="@"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -201,7 +163,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -210,15 +172,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -417,15 +383,16 @@
   <dimension ref="A1:J5"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="39.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="34.97"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="15.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="13.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="12.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="18.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="21.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="17.15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -473,17 +440,14 @@
       <c r="D2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>16</v>
+      <c r="F2" s="2" t="n">
+        <v>45200</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>45184</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>45566</v>
       </c>
       <c r="I2" s="1" t="n">
         <v>365</v>
@@ -493,29 +457,29 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="2" t="n">
+      <c r="A3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="3" t="n">
         <v>70000001327</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>18</v>
+      <c r="C3" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>22</v>
+        <v>15</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>45201</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>45185</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>45567</v>
       </c>
       <c r="I3" s="1" t="n">
         <v>365</v>
@@ -525,11 +489,11 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>24</v>
+      <c r="A4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>2</v>
@@ -538,16 +502,16 @@
         <v>1</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>28</v>
+        <v>18</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>45202</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>45186</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>45568</v>
       </c>
       <c r="I4" s="1" t="n">
         <v>365</v>
@@ -558,34 +522,34 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B5" s="5" t="n">
         <v>970000000041</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>3</v>
+        <v>9741</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>1</v>
+        <v>111</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>33</v>
+        <v>20</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>46299</v>
       </c>
       <c r="I5" s="1" t="n">
-        <v>365</v>
+        <v>100</v>
       </c>
       <c r="J5" s="1" t="n">
-        <v>30</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>